<commit_message>
feat: improve excel write flow and add config-driven settings
- return structured result from write_excel_record and handle locked/write-failed cases in UI

- load runtime defaults from config.toml with safe fallbacks

- add changelog entries for unreleased and recent commits
</commit_message>
<xml_diff>
--- a/data/handcontrol_ui_template.xlsx
+++ b/data/handcontrol_ui_template.xlsx
@@ -196,7 +196,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill/>
     </fill>
@@ -392,6 +392,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -664,7 +669,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -679,6 +684,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1091,7 +1097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="2"/>
   <cols>
     <col width="15.7363636363636" customWidth="1" min="4" max="4"/>
@@ -1187,7 +1193,6 @@
           <t>2026.03.20</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>待确认</t>
@@ -1195,27 +1200,66 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>L39</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>test2</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>x1</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>中、英、越</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>V111.3.5</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>2025.12.03</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>测试通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>LTEST</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>V1.0.0</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>2026.03.20</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>

</xml_diff>

<commit_message>
feat: add attachment field across UI preview and excel flow
</commit_message>
<xml_diff>
--- a/data/handcontrol_ui_template.xlsx
+++ b/data/handcontrol_ui_template.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="25600" windowHeight="12430" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -46,13 +46,6 @@
     </font>
     <font>
       <name val="宋体"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
       <charset val="0"/>
       <color rgb="FF0000FF"/>
       <sz val="11"/>
@@ -196,7 +189,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -205,6 +198,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -224,12 +229,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -523,153 +522,153 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -677,14 +676,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1098,11 +1096,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I5"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="4"/>
   <cols>
     <col width="15.7363636363636" customWidth="1" min="4" max="4"/>
+    <col width="17.2" customWidth="1" min="5" max="5"/>
     <col width="18.4636363636364" customWidth="1" min="6" max="6"/>
     <col width="17.7636363636364" customWidth="1" min="7" max="7"/>
+    <col width="19.8545454545455" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="57" customFormat="1" customHeight="1" s="1">
@@ -1113,153 +1113,158 @@
       </c>
     </row>
     <row r="2" ht="30" customFormat="1" customHeight="1" s="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>型号</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>logo</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>业务员</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>版本号</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>附图</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>L00TEST</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>通用</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DemoUser</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>中、英</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>V0.0.1</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026.03.20</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>待确认</t>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>L39</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>test2</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>x1</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>中、英、越</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>V111.3.5</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>2025.12.03</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>测试通过</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>L39</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>test2</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>x1</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>中、英、越</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>V111.3.5</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>2025.12.03</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>L50</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>dsa</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>sadasd</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>dsad</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>V108.3.3</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>2025.11.07</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>测试通过</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>LTEST</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>V1.0.0</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>2026.03.20</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>V24.4.2</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>2023.11.07</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>

</xml_diff>

<commit_message>
chore: adjust gitignore and restore data files for public repository
</commit_message>
<xml_diff>
--- a/data/handcontrol_ui_template.xlsx
+++ b/data/handcontrol_ui_template.xlsx
@@ -1095,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="4"/>
   <cols>
     <col width="15.7363636363636" customWidth="1" min="4" max="4"/>
@@ -1241,35 +1241,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>L30</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>V24.4.2</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>2023.11.07</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>待确认</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
docs(specs,data): 同步 backlog 审查记录与模板文件
- 提交 requirements backlog 的阶段整理结果与 code-review 记录

- 提交 handcontrol_ui_template.xlsx 模板更新

- 将 specs/ui-reactor/new_uigemini.py 加入 .gitignore，避免原型稿进入后续提交

影响范围:

- specs/requirements-backlog.md 与 specs/code-review/*

- data/handcontrol_ui_template.xlsx

- .gitignore

验证:

- 核对暂存文件仅包含 backlog、code-review、xlsx 与 ignore 规则

- tests/test_app_preview_cache.py 与 tests/test_app_quick_locate.py 仍保留在工作区，未纳入本次提交
</commit_message>
<xml_diff>
--- a/data/handcontrol_ui_template.xlsx
+++ b/data/handcontrol_ui_template.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -184,6 +184,13 @@
     <font>
       <name val="宋体"/>
       <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -668,7 +675,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -683,6 +690,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1095,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="4"/>
   <cols>
     <col width="15.7363636363636" customWidth="1" min="4" max="4"/>
@@ -1211,17 +1219,17 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>dsa</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>sadasd</t>
+          <t>111</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>dsad</t>
+          <t>中、英</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -1234,10 +1242,51 @@
           <t>2025.11.07</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n"/>
+      <c r="H4" s="7" t="inlineStr"/>
       <c r="I4" s="7" t="inlineStr">
         <is>
           <t>测试通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>L50</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>test2</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>x1</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>中、英、越</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>V39.3.1_5</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>2026.04.17</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>待确认</t>
         </is>
       </c>
     </row>

</xml_diff>